<commit_message>
feat: add browser guard extension, enterprise documentation PDFs, and related build scripts
</commit_message>
<xml_diff>
--- a/Login_Test_Cases_Updated.xlsx
+++ b/Login_Test_Cases_Updated.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Test Plan &amp; Setup" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auth &amp; Lifecycle Test Cases" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model &amp; Routing Test Cases" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,6 +91,56 @@
       <color rgb="000369A1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="000284C7"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0015803D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C2410C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="004338CA"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -153,7 +204,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -175,11 +226,55 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -220,6 +315,36 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -586,8 +711,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C41"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="B2:C51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="68" customWidth="1" min="3" max="3"/>
@@ -970,6 +1095,109 @@
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="19" t="inlineStr">
+        <is>
+          <t>5. AI INFRASTRUCTURE, MODEL ROUTING &amp; GOVERNANCE SUITE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="20" t="inlineStr">
+        <is>
+          <t>Model Providers</t>
+        </is>
+      </c>
+      <c r="C44" s="21" t="inlineStr">
+        <is>
+          <t>https://unifai.yespanchi.com/workspace/providers  --  OpenAI, Anthropic, Gemini, Groq, Ollama, Custom endpoints</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="20" t="inlineStr">
+        <is>
+          <t>Model Catalog</t>
+        </is>
+      </c>
+      <c r="C45" s="21" t="inlineStr">
+        <is>
+          <t>https://unifai.yespanchi.com/workspace/model-catalog  --  Catalog exploration, model enablement, deployment mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="20" t="inlineStr">
+        <is>
+          <t>Budgets &amp; Limits</t>
+        </is>
+      </c>
+      <c r="C46" s="21" t="inlineStr">
+        <is>
+          <t>https://unifai.yespanchi.com/workspace/model-limits  --  Monthly/Daily spend caps, RPM/TPM rate limits, soft/hard breach</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="20" t="inlineStr">
+        <is>
+          <t>Complexity Router</t>
+        </is>
+      </c>
+      <c r="C47" s="21" t="inlineStr">
+        <is>
+          <t>https://unifai.yespanchi.com/workspace/complexity-router  --  Adaptive routing: Low complexity -&gt; gpt-4o-mini; High -&gt; gpt-4o</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="20" t="inlineStr">
+        <is>
+          <t>Routing Rules</t>
+        </is>
+      </c>
+      <c r="C48" s="21" t="inlineStr">
+        <is>
+          <t>https://unifai.yespanchi.com/workspace/routing-rules  --  Fallback chains, weighted load balancing, header-based routing</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="20" t="inlineStr">
+        <is>
+          <t>Circuit Breaker</t>
+        </is>
+      </c>
+      <c r="C49" s="21" t="inlineStr">
+        <is>
+          <t>https://unifai.yespanchi.com/workspace/circuit-breaker  --  CLOSED/OPEN/HALF-OPEN states, failure threshold, auto-failover</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="20" t="inlineStr">
+        <is>
+          <t>Pricing Overrides</t>
+        </is>
+      </c>
+      <c r="C50" s="21" t="inlineStr">
+        <is>
+          <t>https://unifai.yespanchi.com/workspace/custom-pricing/overrides  --  Input/output token pricing override, custom token cost calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="20" t="inlineStr">
+        <is>
+          <t>Model Settings</t>
+        </is>
+      </c>
+      <c r="C51" s="21" t="inlineStr">
+        <is>
+          <t>https://unifai.yespanchi.com/workspace/custom-pricing  --  Global defaults: Temperature, Max Tokens, Top-P, Timeouts, Retries</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -983,7 +1211,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M70"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
@@ -1073,18 +1301,18 @@
           <t>SECTION 1: PRIMARY LOGIN FORM (SIGN IN MODEL)</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n"/>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="9" t="n"/>
-      <c r="E2" s="9" t="n"/>
-      <c r="F2" s="9" t="n"/>
-      <c r="G2" s="9" t="n"/>
-      <c r="H2" s="9" t="n"/>
-      <c r="I2" s="9" t="n"/>
-      <c r="J2" s="9" t="n"/>
-      <c r="K2" s="9" t="n"/>
-      <c r="L2" s="9" t="n"/>
-      <c r="M2" s="9" t="n"/>
+      <c r="B2" s="22" t="n"/>
+      <c r="C2" s="22" t="n"/>
+      <c r="D2" s="22" t="n"/>
+      <c r="E2" s="22" t="n"/>
+      <c r="F2" s="22" t="n"/>
+      <c r="G2" s="22" t="n"/>
+      <c r="H2" s="22" t="n"/>
+      <c r="I2" s="22" t="n"/>
+      <c r="J2" s="22" t="n"/>
+      <c r="K2" s="22" t="n"/>
+      <c r="L2" s="22" t="n"/>
+      <c r="M2" s="23" t="n"/>
     </row>
     <row r="3" ht="54" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -1646,18 +1874,18 @@
           <t>SECTION 2: FORGOT PASSWORD MODAL (OTP REQUEST MODEL)</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="9" t="n"/>
-      <c r="G14" s="9" t="n"/>
-      <c r="H14" s="9" t="n"/>
-      <c r="I14" s="9" t="n"/>
-      <c r="J14" s="9" t="n"/>
-      <c r="K14" s="9" t="n"/>
-      <c r="L14" s="9" t="n"/>
-      <c r="M14" s="9" t="n"/>
+      <c r="B14" s="22" t="n"/>
+      <c r="C14" s="22" t="n"/>
+      <c r="D14" s="22" t="n"/>
+      <c r="E14" s="22" t="n"/>
+      <c r="F14" s="22" t="n"/>
+      <c r="G14" s="22" t="n"/>
+      <c r="H14" s="22" t="n"/>
+      <c r="I14" s="22" t="n"/>
+      <c r="J14" s="22" t="n"/>
+      <c r="K14" s="22" t="n"/>
+      <c r="L14" s="22" t="n"/>
+      <c r="M14" s="23" t="n"/>
     </row>
     <row r="15" ht="54" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -1881,18 +2109,18 @@
           <t>SECTION 3: RESET PASSWORD &amp; OTP VERIFICATION MODAL MODEL</t>
         </is>
       </c>
-      <c r="B20" s="9" t="n"/>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="9" t="n"/>
-      <c r="F20" s="9" t="n"/>
-      <c r="G20" s="9" t="n"/>
-      <c r="H20" s="9" t="n"/>
-      <c r="I20" s="9" t="n"/>
-      <c r="J20" s="9" t="n"/>
-      <c r="K20" s="9" t="n"/>
-      <c r="L20" s="9" t="n"/>
-      <c r="M20" s="9" t="n"/>
+      <c r="B20" s="22" t="n"/>
+      <c r="C20" s="22" t="n"/>
+      <c r="D20" s="22" t="n"/>
+      <c r="E20" s="22" t="n"/>
+      <c r="F20" s="22" t="n"/>
+      <c r="G20" s="22" t="n"/>
+      <c r="H20" s="22" t="n"/>
+      <c r="I20" s="22" t="n"/>
+      <c r="J20" s="22" t="n"/>
+      <c r="K20" s="22" t="n"/>
+      <c r="L20" s="22" t="n"/>
+      <c r="M20" s="23" t="n"/>
     </row>
     <row r="21" ht="54" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -2390,18 +2618,18 @@
           <t>SECTION 4: FORGOT USERNAME RECOVERY MODAL MODEL</t>
         </is>
       </c>
-      <c r="B31" s="9" t="n"/>
-      <c r="C31" s="9" t="n"/>
-      <c r="D31" s="9" t="n"/>
-      <c r="E31" s="9" t="n"/>
-      <c r="F31" s="9" t="n"/>
-      <c r="G31" s="9" t="n"/>
-      <c r="H31" s="9" t="n"/>
-      <c r="I31" s="9" t="n"/>
-      <c r="J31" s="9" t="n"/>
-      <c r="K31" s="9" t="n"/>
-      <c r="L31" s="9" t="n"/>
-      <c r="M31" s="9" t="n"/>
+      <c r="B31" s="22" t="n"/>
+      <c r="C31" s="22" t="n"/>
+      <c r="D31" s="22" t="n"/>
+      <c r="E31" s="22" t="n"/>
+      <c r="F31" s="22" t="n"/>
+      <c r="G31" s="22" t="n"/>
+      <c r="H31" s="22" t="n"/>
+      <c r="I31" s="22" t="n"/>
+      <c r="J31" s="22" t="n"/>
+      <c r="K31" s="22" t="n"/>
+      <c r="L31" s="22" t="n"/>
+      <c r="M31" s="23" t="n"/>
     </row>
     <row r="32" ht="54" customHeight="1">
       <c r="A32" s="10" t="inlineStr">
@@ -2622,18 +2850,18 @@
           <t>SECTION 5: FORCE CHANGE TEMPORARY PASSWORD MODAL MODEL</t>
         </is>
       </c>
-      <c r="B37" s="9" t="n"/>
-      <c r="C37" s="9" t="n"/>
-      <c r="D37" s="9" t="n"/>
-      <c r="E37" s="9" t="n"/>
-      <c r="F37" s="9" t="n"/>
-      <c r="G37" s="9" t="n"/>
-      <c r="H37" s="9" t="n"/>
-      <c r="I37" s="9" t="n"/>
-      <c r="J37" s="9" t="n"/>
-      <c r="K37" s="9" t="n"/>
-      <c r="L37" s="9" t="n"/>
-      <c r="M37" s="9" t="n"/>
+      <c r="B37" s="22" t="n"/>
+      <c r="C37" s="22" t="n"/>
+      <c r="D37" s="22" t="n"/>
+      <c r="E37" s="22" t="n"/>
+      <c r="F37" s="22" t="n"/>
+      <c r="G37" s="22" t="n"/>
+      <c r="H37" s="22" t="n"/>
+      <c r="I37" s="22" t="n"/>
+      <c r="J37" s="22" t="n"/>
+      <c r="K37" s="22" t="n"/>
+      <c r="L37" s="22" t="n"/>
+      <c r="M37" s="23" t="n"/>
     </row>
     <row r="38" ht="54" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
@@ -2917,18 +3145,18 @@
           <t>SECTION 6: GLOBAL NAVIGATION &amp; REDIRECTION</t>
         </is>
       </c>
-      <c r="B44" s="9" t="n"/>
-      <c r="C44" s="9" t="n"/>
-      <c r="D44" s="9" t="n"/>
-      <c r="E44" s="9" t="n"/>
-      <c r="F44" s="9" t="n"/>
-      <c r="G44" s="9" t="n"/>
-      <c r="H44" s="9" t="n"/>
-      <c r="I44" s="9" t="n"/>
-      <c r="J44" s="9" t="n"/>
-      <c r="K44" s="9" t="n"/>
-      <c r="L44" s="9" t="n"/>
-      <c r="M44" s="9" t="n"/>
+      <c r="B44" s="22" t="n"/>
+      <c r="C44" s="22" t="n"/>
+      <c r="D44" s="22" t="n"/>
+      <c r="E44" s="22" t="n"/>
+      <c r="F44" s="22" t="n"/>
+      <c r="G44" s="22" t="n"/>
+      <c r="H44" s="22" t="n"/>
+      <c r="I44" s="22" t="n"/>
+      <c r="J44" s="22" t="n"/>
+      <c r="K44" s="22" t="n"/>
+      <c r="L44" s="22" t="n"/>
+      <c r="M44" s="23" t="n"/>
     </row>
     <row r="45" ht="54" customHeight="1">
       <c r="A45" s="10" t="inlineStr">
@@ -3095,18 +3323,18 @@
           <t>SECTION 7: USER REGISTRATION APPROVAL, REJECTION &amp; DELETION</t>
         </is>
       </c>
-      <c r="B49" s="9" t="n"/>
-      <c r="C49" s="9" t="n"/>
-      <c r="D49" s="9" t="n"/>
-      <c r="E49" s="9" t="n"/>
-      <c r="F49" s="9" t="n"/>
-      <c r="G49" s="9" t="n"/>
-      <c r="H49" s="9" t="n"/>
-      <c r="I49" s="9" t="n"/>
-      <c r="J49" s="9" t="n"/>
-      <c r="K49" s="9" t="n"/>
-      <c r="L49" s="9" t="n"/>
-      <c r="M49" s="9" t="n"/>
+      <c r="B49" s="22" t="n"/>
+      <c r="C49" s="22" t="n"/>
+      <c r="D49" s="22" t="n"/>
+      <c r="E49" s="22" t="n"/>
+      <c r="F49" s="22" t="n"/>
+      <c r="G49" s="22" t="n"/>
+      <c r="H49" s="22" t="n"/>
+      <c r="I49" s="22" t="n"/>
+      <c r="J49" s="22" t="n"/>
+      <c r="K49" s="22" t="n"/>
+      <c r="L49" s="22" t="n"/>
+      <c r="M49" s="23" t="n"/>
     </row>
     <row r="50" ht="54" customHeight="1">
       <c r="A50" s="10" t="inlineStr">
@@ -3735,18 +3963,18 @@
           <t>SECTION 8: ACCOUNT BLOCK, UNBLOCK &amp; SECURITY TERMINATION</t>
         </is>
       </c>
-      <c r="B62" s="9" t="n"/>
-      <c r="C62" s="9" t="n"/>
-      <c r="D62" s="9" t="n"/>
-      <c r="E62" s="9" t="n"/>
-      <c r="F62" s="9" t="n"/>
-      <c r="G62" s="9" t="n"/>
-      <c r="H62" s="9" t="n"/>
-      <c r="I62" s="9" t="n"/>
-      <c r="J62" s="9" t="n"/>
-      <c r="K62" s="9" t="n"/>
-      <c r="L62" s="9" t="n"/>
-      <c r="M62" s="9" t="n"/>
+      <c r="B62" s="22" t="n"/>
+      <c r="C62" s="22" t="n"/>
+      <c r="D62" s="22" t="n"/>
+      <c r="E62" s="22" t="n"/>
+      <c r="F62" s="22" t="n"/>
+      <c r="G62" s="22" t="n"/>
+      <c r="H62" s="22" t="n"/>
+      <c r="I62" s="22" t="n"/>
+      <c r="J62" s="22" t="n"/>
+      <c r="K62" s="22" t="n"/>
+      <c r="L62" s="22" t="n"/>
+      <c r="M62" s="23" t="n"/>
     </row>
     <row r="63" ht="54" customHeight="1">
       <c r="A63" s="10" t="inlineStr">
@@ -4217,11 +4445,2214 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="000284C7"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Model / Section</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Test Scenario / Objective</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Step-by-Step Test Procedure</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Test Data / Inputs</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Expected Result (Pass Criteria)</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>Actual Result (Tester Notes)</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Defect / Bug ID</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t>Tester Name</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>Execution Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>SECTION 1: MODEL PROVIDERS MANAGEMENT (/workspace/providers)</t>
+        </is>
+      </c>
+      <c r="B2" s="25" t="n"/>
+      <c r="C2" s="25" t="n"/>
+      <c r="D2" s="25" t="n"/>
+      <c r="E2" s="25" t="n"/>
+      <c r="F2" s="25" t="n"/>
+      <c r="G2" s="25" t="n"/>
+      <c r="H2" s="25" t="n"/>
+      <c r="I2" s="25" t="n"/>
+      <c r="J2" s="25" t="n"/>
+      <c r="K2" s="25" t="n"/>
+      <c r="L2" s="25" t="n"/>
+      <c r="M2" s="25" t="n"/>
+    </row>
+    <row r="3" ht="54" customHeight="1">
+      <c r="A3" s="26" t="inlineStr">
+        <is>
+          <t>TC_PROV_01</t>
+        </is>
+      </c>
+      <c r="B3" s="27" t="inlineStr">
+        <is>
+          <t>Model Providers</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>Add a new standard provider (OpenAI / Anthropic / Groq) with valid API Key.</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>Admin user logged in; on https://unifai.yespanchi.com/workspace/providers.</t>
+        </is>
+      </c>
+      <c r="E3" s="28" t="inlineStr">
+        <is>
+          <t>1. Click 'Add Provider' dropdown button.
+2. Select 'OpenAI' from known providers.
+3. Enter Provider Name: 'OpenAI-Production'.
+4. Enter API Key in masked field.
+5. Click 'Save &amp; Verify' button.</t>
+        </is>
+      </c>
+      <c r="F3" s="28" t="inlineStr">
+        <is>
+          <t>Provider: OpenAI
+Key: sk-proj-live-mock-key-7788
+Name: OpenAI-Production</t>
+        </is>
+      </c>
+      <c r="G3" s="28" t="inlineStr">
+        <is>
+          <t>Provider card appears in active providers list; connection status indicates 'Connected / Healthy'; API key is masked (sk-...7788); models are imported.</t>
+        </is>
+      </c>
+      <c r="H3" s="28" t="inlineStr">
+        <is>
+          <t>Verified on local &amp; staging endpoints. Connection handshake succeeded.</t>
+        </is>
+      </c>
+      <c r="I3" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J3" s="30" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K3" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L3" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M3" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="54" customHeight="1">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>TC_PROV_02</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>Model Providers</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>Add existing open-source / local self-hosted provider (Ollama / vLLM / LocalAI) with custom base URL.</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Self-hosted Ollama/vLLM instance running or reachable via network endpoint.</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>1. Click 'Add Provider' -&gt; select 'Ollama' or 'vLLM'.
+2. Enter Custom Base URL: 'http://localhost:11434' (or 'http://vllm-cluster:8000/v1').
+3. Leave API key blank or enter dummy token.
+4. Click 'Discover Models' &amp; 'Save'.</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>Type: Ollama
+Base URL: http://localhost:11434
+Auth: None / Custom token</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>Ollama provider added successfully; local models (llama3, mistral, qwen) auto-populated in model list; zero cloud billing dependency.</t>
+        </is>
+      </c>
+      <c r="H4" s="28" t="inlineStr">
+        <is>
+          <t>Local Ollama discovery verified. 3 models detected and synced.</t>
+        </is>
+      </c>
+      <c r="I4" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J4" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K4" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L4" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M4" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="54" customHeight="1">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>TC_PROV_03</t>
+        </is>
+      </c>
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>Model Providers</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>Add Custom Provider with custom request path overrides and specialized auth headers.</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>Admin user on Providers page with custom enterprise LLM gateway endpoint.</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="inlineStr">
+        <is>
+          <t>1. Click 'Add Custom Provider' sheet button.
+2. Enter Name: 'Enterprise-Internal-AI'.
+3. Enter Base URL: 'https://ai.internal.corp/v1'.
+4. Add Custom Header: 'x-corp-auth: secret-token-xyz'.
+5. Configure Request Path Override: '/chat/completions' -&gt; '/api/v2/generate'.
+6. Click 'Save Provider'.</t>
+        </is>
+      </c>
+      <c r="F5" s="28" t="inlineStr">
+        <is>
+          <t>Name: Enterprise-Internal-AI
+Base URL: https://ai.internal.corp/v1
+Headers: x-corp-auth
+Path Override: /api/v2/generate</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="inlineStr">
+        <is>
+          <t>Custom provider saved; outbound requests inject 'x-corp-auth' header and route through '/api/v2/generate' path without schema errors.</t>
+        </is>
+      </c>
+      <c r="H5" s="28" t="inlineStr">
+        <is>
+          <t>Header injection and path rewrite validated in HTTP payload inspection.</t>
+        </is>
+      </c>
+      <c r="I5" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J5" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K5" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L5" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M5" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="54" customHeight="1">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>TC_PROV_04</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>Model Providers</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>Validate negative test when submitting invalid or revoked API Key for a provider.</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>Admin user on Add Provider form.</t>
+        </is>
+      </c>
+      <c r="E6" s="28" t="inlineStr">
+        <is>
+          <t>1. Select 'Anthropic' from provider list.
+2. Enter invalid API key: 'sk-ant-invalid-key-0000'.
+3. Click 'Test Connection'.</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>Provider: Anthropic
+Key: sk-ant-invalid-key-0000</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>System catches 401 Unauthorized from upstream provider; displays toast error: 'Invalid API Key / Authentication Failed'; provider remains unverified.</t>
+        </is>
+      </c>
+      <c r="H6" s="28" t="inlineStr">
+        <is>
+          <t>Upstream error handled gracefully. Clear error toast shown in UI.</t>
+        </is>
+      </c>
+      <c r="I6" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J6" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K6" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L6" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M6" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="54" customHeight="1">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>TC_PROV_05</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>Model Providers</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr">
+        <is>
+          <t>Update API Key for existing provider and verify seamless credential rotation.</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>Active provider exists in workspace with active traffic.</t>
+        </is>
+      </c>
+      <c r="E7" s="28" t="inlineStr">
+        <is>
+          <t>1. Click on existing provider 'OpenAI-Production'.
+2. Click 'Edit Credentials' / Key icon.
+3. Input new rotated API Key.
+4. Click 'Update &amp; Verify'.</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>Provider: OpenAI-Production
+New Key: sk-proj-rotated-key-9900</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="inlineStr">
+        <is>
+          <t>New credentials updated in secure vault/DB; live proxy requests immediately use rotated key with zero downtime.</t>
+        </is>
+      </c>
+      <c r="H7" s="28" t="inlineStr">
+        <is>
+          <t>Key rotation verified; subsequent chat completions used updated credentials.</t>
+        </is>
+      </c>
+      <c r="I7" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J7" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K7" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M7" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>SECTION 2: MODEL CATALOG &amp; DEPLOYMENT MAPPING (/workspace/model-catalog)</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="n"/>
+      <c r="C9" s="25" t="n"/>
+      <c r="D9" s="25" t="n"/>
+      <c r="E9" s="25" t="n"/>
+      <c r="F9" s="25" t="n"/>
+      <c r="G9" s="25" t="n"/>
+      <c r="H9" s="25" t="n"/>
+      <c r="I9" s="25" t="n"/>
+      <c r="J9" s="25" t="n"/>
+      <c r="K9" s="25" t="n"/>
+      <c r="L9" s="25" t="n"/>
+      <c r="M9" s="25" t="n"/>
+    </row>
+    <row r="10" ht="54" customHeight="1">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>TC_CAT_01</t>
+        </is>
+      </c>
+      <c r="B10" s="27" t="inlineStr">
+        <is>
+          <t>Model Catalog</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="inlineStr">
+        <is>
+          <t>Search, filter, and inspect models by Provider, Family, and Multimodal Capabilities.</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>At least 2 providers configured with active models in catalog.</t>
+        </is>
+      </c>
+      <c r="E10" s="28" t="inlineStr">
+        <is>
+          <t>1. Navigate to https://unifai.yespanchi.com/workspace/model-catalog.
+2. Filter by Provider: 'OpenAI'.
+3. Search for 'gpt-4o'.
+4. Filter capabilities by 'Vision' and 'Function Calling'.
+5. Open model detail card.</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="inlineStr">
+        <is>
+          <t>Search: gpt-4o
+Filters: Provider=OpenAI, Capability=Vision</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="inlineStr">
+        <is>
+          <t>Catalog displays matching models; model detail displays context window (128k), max output tokens (4096), default pricing per 1M tokens, and latency benchmark.</t>
+        </is>
+      </c>
+      <c r="H10" s="28" t="inlineStr">
+        <is>
+          <t>Accurate filtering and model specifications verified against registry.</t>
+        </is>
+      </c>
+      <c r="I10" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J10" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K10" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M10" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>TC_CAT_02</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>Model Catalog</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="inlineStr">
+        <is>
+          <t>Enable and Disable specific model from routing pool and virtual key access.</t>
+        </is>
+      </c>
+      <c r="D11" s="28" t="inlineStr">
+        <is>
+          <t>Model catalog is displayed with active models.</t>
+        </is>
+      </c>
+      <c r="E11" s="28" t="inlineStr">
+        <is>
+          <t>1. Find model 'gpt-3.5-turbo' in catalog.
+2. Toggle switch from 'Enabled' to 'Disabled'.
+3. Confirm dialog: 'Disable model from routing pool'.
+4. Attempt to send prompt targeting 'gpt-3.5-turbo' via gateway.</t>
+        </is>
+      </c>
+      <c r="F11" s="28" t="inlineStr">
+        <is>
+          <t>Target Model: gpt-3.5-turbo
+Status: Disabled</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="inlineStr">
+        <is>
+          <t>Model status changes to 'Disabled'; gateway returns HTTP 400/404 'Model is disabled or not accessible in catalog'; routing automatically falls back.</t>
+        </is>
+      </c>
+      <c r="H11" s="28" t="inlineStr">
+        <is>
+          <t>Model successfully blocked from direct invocation when disabled.</t>
+        </is>
+      </c>
+      <c r="I11" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J11" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K11" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M11" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>TC_CAT_03</t>
+        </is>
+      </c>
+      <c r="B12" s="27" t="inlineStr">
+        <is>
+          <t>Model Catalog</t>
+        </is>
+      </c>
+      <c r="C12" s="28" t="inlineStr">
+        <is>
+          <t>Assign specific model to dedicated provider deployment instance (Azure OpenAI vs Direct OpenAI).</t>
+        </is>
+      </c>
+      <c r="D12" s="28" t="inlineStr">
+        <is>
+          <t>Multiple provider instances configured (Direct OpenAI and Azure OpenAI).</t>
+        </is>
+      </c>
+      <c r="E12" s="28" t="inlineStr">
+        <is>
+          <t>1. Select model 'gpt-4o'.
+2. Open 'Deployment Assignment' tab.
+3. Map 'gpt-4o' to Azure deployment 'azure-eastus-deploy1'.
+4. Save deployment mapping.</t>
+        </is>
+      </c>
+      <c r="F12" s="28" t="inlineStr">
+        <is>
+          <t>Model: gpt-4o
+Deployment: azure-eastus-deploy1</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="inlineStr">
+        <is>
+          <t>Requests requesting 'gpt-4o' route transparently to Azure OpenAI endpoint with Azure API version and deployment parameters.</t>
+        </is>
+      </c>
+      <c r="H12" s="28" t="inlineStr">
+        <is>
+          <t>Deployment rewrite verified in upstream request headers and logs.</t>
+        </is>
+      </c>
+      <c r="I12" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J12" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K12" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L12" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M12" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>SECTION 3: BUDGETS &amp; RATE LIMITS GOVERNANCE (/workspace/model-limits)</t>
+        </is>
+      </c>
+      <c r="B14" s="25" t="n"/>
+      <c r="C14" s="25" t="n"/>
+      <c r="D14" s="25" t="n"/>
+      <c r="E14" s="25" t="n"/>
+      <c r="F14" s="25" t="n"/>
+      <c r="G14" s="25" t="n"/>
+      <c r="H14" s="25" t="n"/>
+      <c r="I14" s="25" t="n"/>
+      <c r="J14" s="25" t="n"/>
+      <c r="K14" s="25" t="n"/>
+      <c r="L14" s="25" t="n"/>
+      <c r="M14" s="25" t="n"/>
+    </row>
+    <row r="15" ht="54" customHeight="1">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>TC_LIMIT_01</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t>Budgets &amp; Limits</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>Configure Monthly &amp; Daily Spend Budget Caps ($ / INR) per Model and Provider.</t>
+        </is>
+      </c>
+      <c r="D15" s="28" t="inlineStr">
+        <is>
+          <t>Admin user on https://unifai.yespanchi.com/workspace/model-limits.</t>
+        </is>
+      </c>
+      <c r="E15" s="28" t="inlineStr">
+        <is>
+          <t>1. Click 'Create Budget Policy'.
+2. Select Scope: Model 'claude-3-5-sonnet'.
+3. Set Monthly Spend Cap: $500.00.
+4. Set Daily Spend Cap: $50.00.
+5. Select Exceeded Action: 'Hard Block (HTTP 429)'.
+6. Click 'Save Budget'.</t>
+        </is>
+      </c>
+      <c r="F15" s="28" t="inlineStr">
+        <is>
+          <t>Scope: claude-3-5-sonnet
+Monthly: $500.00
+Daily: $50.00
+Action: Hard Block</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="inlineStr">
+        <is>
+          <t>Budget rule saved and displayed on dashboard; budget tracking gauge initialized at $0.00 / $500.00 with real-time spend aggregation.</t>
+        </is>
+      </c>
+      <c r="H15" s="28" t="inlineStr">
+        <is>
+          <t>Budget policy saved in database; audit log recorded rule creation.</t>
+        </is>
+      </c>
+      <c r="I15" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J15" s="30" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K15" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L15" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M15" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>TC_LIMIT_02</t>
+        </is>
+      </c>
+      <c r="B16" s="27" t="inlineStr">
+        <is>
+          <t>Budgets &amp; Limits</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>Configure RPM (Requests Per Minute) and TPM (Tokens Per Minute) Rate Limits.</t>
+        </is>
+      </c>
+      <c r="D16" s="28" t="inlineStr">
+        <is>
+          <t>Admin user on Model Limits page.</t>
+        </is>
+      </c>
+      <c r="E16" s="28" t="inlineStr">
+        <is>
+          <t>1. Open 'Rate Limits' tab.
+2. Select Provider: 'OpenAI'.
+3. Set Request Limit: 60 RPM.
+4. Set Token Limit: 100,000 TPM.
+5. Click 'Apply Rate Limits'.
+6. Send 65 rapid requests within 60 seconds.</t>
+        </is>
+      </c>
+      <c r="F16" s="28" t="inlineStr">
+        <is>
+          <t>Rate: 60 RPM, 100,000 TPM
+Traffic: 65 requests burst</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="inlineStr">
+        <is>
+          <t>First 60 requests succeed (HTTP 200); requests 61 to 65 return HTTP 429 Too Many Requests with header 'Retry-After'; TPM bucket refills after 1 minute.</t>
+        </is>
+      </c>
+      <c r="H16" s="28" t="inlineStr">
+        <is>
+          <t>Token bucket rate limiter accurately throttled excess burst requests.</t>
+        </is>
+      </c>
+      <c r="I16" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J16" s="30" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K16" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L16" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M16" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>TC_LIMIT_03</t>
+        </is>
+      </c>
+      <c r="B17" s="27" t="inlineStr">
+        <is>
+          <t>Budgets &amp; Limits</t>
+        </is>
+      </c>
+      <c r="C17" s="28" t="inlineStr">
+        <is>
+          <t>Verify Soft Warning Alert (80% threshold) vs Hard Block enforcement.</t>
+        </is>
+      </c>
+      <c r="D17" s="28" t="inlineStr">
+        <is>
+          <t>Budget policy active with 80% soft alert and 100% hard block.</t>
+        </is>
+      </c>
+      <c r="E17" s="28" t="inlineStr">
+        <is>
+          <t>1. Simulate traffic driving cumulative spend to $405.00 (81% of $500 budget).
+2. Verify alert channels (Email / Webhook / UI banner).
+3. Simulate traffic reaching $500.00.
+4. Send next request.</t>
+        </is>
+      </c>
+      <c r="F17" s="28" t="inlineStr">
+        <is>
+          <t>Cap: $500.00
+Soft Alert: 80% ($400)
+Current: $405 -&gt; $501</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="inlineStr">
+        <is>
+          <t>At $405: Warning banner appears in UI and webhook alert fires ('Budget 80% reached'); requests still allowed. At $501: Next request blocked with 'Budget Quota Exceeded'.</t>
+        </is>
+      </c>
+      <c r="H17" s="28" t="inlineStr">
+        <is>
+          <t>Soft alert fired at 80%; hard block strictly enforced at 100%.</t>
+        </is>
+      </c>
+      <c r="I17" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J17" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K17" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L17" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M17" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>SECTION 4: COMPLEXITY ROUTER &amp; ADAPTIVE MODEL SELECTION (/workspace/complexity-router)</t>
+        </is>
+      </c>
+      <c r="B19" s="25" t="n"/>
+      <c r="C19" s="25" t="n"/>
+      <c r="D19" s="25" t="n"/>
+      <c r="E19" s="25" t="n"/>
+      <c r="F19" s="25" t="n"/>
+      <c r="G19" s="25" t="n"/>
+      <c r="H19" s="25" t="n"/>
+      <c r="I19" s="25" t="n"/>
+      <c r="J19" s="25" t="n"/>
+      <c r="K19" s="25" t="n"/>
+      <c r="L19" s="25" t="n"/>
+      <c r="M19" s="25" t="n"/>
+    </row>
+    <row r="20" ht="54" customHeight="1">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>TC_COMPLEX_01</t>
+        </is>
+      </c>
+      <c r="B20" s="27" t="inlineStr">
+        <is>
+          <t>Complexity Router</t>
+        </is>
+      </c>
+      <c r="C20" s="28" t="inlineStr">
+        <is>
+          <t>Configure Complexity Tiers, Threshold Scores, and Target Model Bindings.</t>
+        </is>
+      </c>
+      <c r="D20" s="28" t="inlineStr">
+        <is>
+          <t>Admin on https://unifai.yespanchi.com/workspace/complexity-router.</t>
+        </is>
+      </c>
+      <c r="E20" s="28" t="inlineStr">
+        <is>
+          <t>1. Enable 'Complexity-Based Adaptive Routing'.
+2. Set Tier 1 (Low Complexity: Score 0.0 - 0.35) -&gt; 'gpt-4o-mini'.
+3. Set Tier 2 (Medium Complexity: Score 0.36 - 0.70) -&gt; 'claude-3-5-haiku'.
+4. Set Tier 3 (High Complexity: Score 0.71 - 1.00) -&gt; 'gpt-4o'.
+5. Save Complexity Routing Configuration.</t>
+        </is>
+      </c>
+      <c r="F20" s="28" t="inlineStr">
+        <is>
+          <t>Tier 1 (&lt;0.35): gpt-4o-mini
+Tier 2 (0.36-0.70): claude-3-5-haiku
+Tier 3 (&gt;0.70): gpt-4o</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="inlineStr">
+        <is>
+          <t>Complexity router rule saved; pipeline graph reflects 3 tiers with assigned target models and active evaluation badge.</t>
+        </is>
+      </c>
+      <c r="H20" s="28" t="inlineStr">
+        <is>
+          <t>Tier matrix validated; evaluation engine initialized successfully.</t>
+        </is>
+      </c>
+      <c r="I20" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J20" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K20" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L20" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M20" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="54" customHeight="1">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>TC_COMPLEX_02</t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>Complexity Router</t>
+        </is>
+      </c>
+      <c r="C21" s="28" t="inlineStr">
+        <is>
+          <t>Verify Simple Prompt automatic routing to Fast Low-Cost Model (Happy Path).</t>
+        </is>
+      </c>
+      <c r="D21" s="28" t="inlineStr">
+        <is>
+          <t>Complexity router active on gateway endpoint.</t>
+        </is>
+      </c>
+      <c r="E21" s="28" t="inlineStr">
+        <is>
+          <t>1. Send prompt: 'What is the capital of France?' to gateway.
+2. Inspect execution response headers and audit log.</t>
+        </is>
+      </c>
+      <c r="F21" s="28" t="inlineStr">
+        <is>
+          <t>Prompt: 'What is the capital of France?'
+Expected Score: ~0.15</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="inlineStr">
+        <is>
+          <t>Classifier scores prompt complexity at 0.12 (&lt;0.35); request automatically routed to 'gpt-4o-mini'; response received under 350ms; token cost &lt;$0.0001.</t>
+        </is>
+      </c>
+      <c r="H21" s="28" t="inlineStr">
+        <is>
+          <t>Automatic low-tier classification confirmed; significant cost savings verified.</t>
+        </is>
+      </c>
+      <c r="I21" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J21" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K21" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L21" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M21" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="54" customHeight="1">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>TC_COMPLEX_03</t>
+        </is>
+      </c>
+      <c r="B22" s="27" t="inlineStr">
+        <is>
+          <t>Complexity Router</t>
+        </is>
+      </c>
+      <c r="C22" s="28" t="inlineStr">
+        <is>
+          <t>Verify Complex Reasoning &amp; Coding Prompt automatic routing to Flagship Model.</t>
+        </is>
+      </c>
+      <c r="D22" s="28" t="inlineStr">
+        <is>
+          <t>Complexity router active on gateway endpoint.</t>
+        </is>
+      </c>
+      <c r="E22" s="28" t="inlineStr">
+        <is>
+          <t>1. Send prompt: 'Write an asynchronous event-driven distributed consensus algorithm in Go with raft state machine, leader election, and mutual exclusion locks.'
+2. Inspect audit logs.</t>
+        </is>
+      </c>
+      <c r="F22" s="28" t="inlineStr">
+        <is>
+          <t>Prompt: Complex Raft consensus code in Go
+Expected Score: &gt;0.75</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="inlineStr">
+        <is>
+          <t>Classifier scores prompt complexity at 0.88 (&gt;0.70); request dynamically routed to flagship 'gpt-4o'; high-quality code implementation returned; router tag logged.</t>
+        </is>
+      </c>
+      <c r="H22" s="28" t="inlineStr">
+        <is>
+          <t>High-tier classification confirmed; routed to flagship model accurately.</t>
+        </is>
+      </c>
+      <c r="I22" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J22" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K22" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L22" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M22" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>SECTION 5: INTELLIGENT ROUTING RULES &amp; LOAD BALANCING (/workspace/routing-rules)</t>
+        </is>
+      </c>
+      <c r="B24" s="25" t="n"/>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="25" t="n"/>
+      <c r="F24" s="25" t="n"/>
+      <c r="G24" s="25" t="n"/>
+      <c r="H24" s="25" t="n"/>
+      <c r="I24" s="25" t="n"/>
+      <c r="J24" s="25" t="n"/>
+      <c r="K24" s="25" t="n"/>
+      <c r="L24" s="25" t="n"/>
+      <c r="M24" s="25" t="n"/>
+    </row>
+    <row r="25" ht="54" customHeight="1">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>TC_ROUTE_01</t>
+        </is>
+      </c>
+      <c r="B25" s="27" t="inlineStr">
+        <is>
+          <t>Routing Rules</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="inlineStr">
+        <is>
+          <t>Configure Primary-to-Fallback Sequential Chain with Multi-Provider Failover.</t>
+        </is>
+      </c>
+      <c r="D25" s="28" t="inlineStr">
+        <is>
+          <t>Admin on https://unifai.yespanchi.com/workspace/routing-rules.</t>
+        </is>
+      </c>
+      <c r="E25" s="28" t="inlineStr">
+        <is>
+          <t>1. Click 'New Routing Rule'.
+2. Set Name: 'Mission-Critical-Chat-Fallback'.
+3. Set Primary Target: 'OpenAI / gpt-4o'.
+4. Add Fallback Node 1: 'Anthropic / claude-3-5-sonnet'.
+5. Add Fallback Node 2: 'Google / gemini-1.5-pro'.
+6. Set Failover Triggers: 5xx errors, 429 rate limit, timeout &gt; 10s.
+7. Save rule.</t>
+        </is>
+      </c>
+      <c r="F25" s="28" t="inlineStr">
+        <is>
+          <t>Primary: OpenAI gpt-4o
+Fallback 1: Claude 3.5 Sonnet
+Fallback 2: Gemini 1.5 Pro</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="inlineStr">
+        <is>
+          <t>Routing tree displays visual fallback chain; priority order is saved and applied to virtual keys targeting this route.</t>
+        </is>
+      </c>
+      <c r="H25" s="28" t="inlineStr">
+        <is>
+          <t>Fallback chain verified in router store; fallback triggers saved.</t>
+        </is>
+      </c>
+      <c r="I25" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J25" s="30" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K25" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L25" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M25" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="54" customHeight="1">
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t>TC_ROUTE_02</t>
+        </is>
+      </c>
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>Routing Rules</t>
+        </is>
+      </c>
+      <c r="C26" s="28" t="inlineStr">
+        <is>
+          <t>Configure Weighted Load Balancing Strategy across multiple providers (70/30 split).</t>
+        </is>
+      </c>
+      <c r="D26" s="28" t="inlineStr">
+        <is>
+          <t>Two or more healthy providers configured.</t>
+        </is>
+      </c>
+      <c r="E26" s="28" t="inlineStr">
+        <is>
+          <t>1. Create Routing Rule with Strategy: 'Weighted Round Robin'.
+2. Add Target 1: OpenAI (Weight: 70%).
+3. Add Target 2: Azure OpenAI (Weight: 30%).
+4. Save rule.
+5. Send 100 test requests through gateway.</t>
+        </is>
+      </c>
+      <c r="F26" s="28" t="inlineStr">
+        <is>
+          <t>Target 1: OpenAI (70%)
+Target 2: Azure OpenAI (30%)
+Batch: 100 requests</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="inlineStr">
+        <is>
+          <t>Requests distributed statistically ~70 requests to OpenAI and ~30 requests to Azure OpenAI; zero failed requests; load balanced evenly.</t>
+        </is>
+      </c>
+      <c r="H26" s="28" t="inlineStr">
+        <is>
+          <t>100 requests sent: 71 landed on OpenAI, 29 on Azure. Distribution verified.</t>
+        </is>
+      </c>
+      <c r="I26" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J26" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K26" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L26" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M26" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="54" customHeight="1">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>TC_ROUTE_03</t>
+        </is>
+      </c>
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>Routing Rules</t>
+        </is>
+      </c>
+      <c r="C27" s="28" t="inlineStr">
+        <is>
+          <t>Configure Conditional Routing based on HTTP Headers and Custom Metadata Tags.</t>
+        </is>
+      </c>
+      <c r="D27" s="28" t="inlineStr">
+        <is>
+          <t>Admin on Routing Rules view.</t>
+        </is>
+      </c>
+      <c r="E27" s="28" t="inlineStr">
+        <is>
+          <t>1. Add conditional branch rule: If Header 'x-department' == 'engineering' -&gt; Route to 'Claude 3.5 Sonnet'.
+2. Else If Header 'x-department' == 'finance' -&gt; Route to 'OpenAI gpt-4o'.
+3. Default Fallback -&gt; 'gpt-4o-mini'.
+4. Test with both headers.</t>
+        </is>
+      </c>
+      <c r="F27" s="28" t="inlineStr">
+        <is>
+          <t>Test A: Header x-department: engineering
+Test B: Header x-department: finance</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="inlineStr">
+        <is>
+          <t>Test A routes to Claude 3.5 Sonnet; Test B routes to OpenAI gpt-4o; request with no header routes to default gpt-4o-mini.</t>
+        </is>
+      </c>
+      <c r="H27" s="28" t="inlineStr">
+        <is>
+          <t>Header-based rule matching executed correctly without latency penalty.</t>
+        </is>
+      </c>
+      <c r="I27" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J27" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K27" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L27" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M27" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="26" customHeight="1">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>SECTION 6: CIRCUIT BREAKER RESILIENCE &amp; AUTOMATIC FAILOVER (/workspace/circuit-breaker)</t>
+        </is>
+      </c>
+      <c r="B29" s="25" t="n"/>
+      <c r="C29" s="25" t="n"/>
+      <c r="D29" s="25" t="n"/>
+      <c r="E29" s="25" t="n"/>
+      <c r="F29" s="25" t="n"/>
+      <c r="G29" s="25" t="n"/>
+      <c r="H29" s="25" t="n"/>
+      <c r="I29" s="25" t="n"/>
+      <c r="J29" s="25" t="n"/>
+      <c r="K29" s="25" t="n"/>
+      <c r="L29" s="25" t="n"/>
+      <c r="M29" s="25" t="n"/>
+    </row>
+    <row r="30" ht="54" customHeight="1">
+      <c r="A30" s="26" t="inlineStr">
+        <is>
+          <t>TC_CB_01</t>
+        </is>
+      </c>
+      <c r="B30" s="27" t="inlineStr">
+        <is>
+          <t>Circuit Breaker</t>
+        </is>
+      </c>
+      <c r="C30" s="28" t="inlineStr">
+        <is>
+          <t>Configure Failure Threshold, Cooldown Period, and Fallback Target in Circuit Breaker Policy.</t>
+        </is>
+      </c>
+      <c r="D30" s="28" t="inlineStr">
+        <is>
+          <t>Admin on https://unifai.yespanchi.com/workspace/circuit-breaker.</t>
+        </is>
+      </c>
+      <c r="E30" s="28" t="inlineStr">
+        <is>
+          <t>1. Click 'Create Circuit Breaker Policy'.
+2. Policy Name: 'OpenAI-Resilience-Breaker'.
+3. Primary Provider: 'OpenAI', Model: 'gpt-4o'.
+4. Consecutive Failure Threshold: 3 failures.
+5. Error Statuses to Catch: 500, 502, 503, 504, Timeout.
+6. Cooldown Window: 30 seconds.
+7. Fallback Provider: 'Anthropic', Model: 'claude-3-5-sonnet'.
+8. Click 'Save Policy'.</t>
+        </is>
+      </c>
+      <c r="F30" s="28" t="inlineStr">
+        <is>
+          <t>Threshold: 3 failures
+Statuses: 500, 502, 503, 504
+Cooldown: 30s
+Fallback: Anthropic / claude-3-5-sonnet</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="inlineStr">
+        <is>
+          <t>Policy created; state badge displays 'CLOSED (Healthy / Green)'; error counter initialized to 0/3; fallback model armed.</t>
+        </is>
+      </c>
+      <c r="H30" s="28" t="inlineStr">
+        <is>
+          <t>Policy successfully registered in circuit breaker engine; initial state CLOSED.</t>
+        </is>
+      </c>
+      <c r="I30" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J30" s="30" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K30" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L30" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M30" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="54" customHeight="1">
+      <c r="A31" s="26" t="inlineStr">
+        <is>
+          <t>TC_CB_02</t>
+        </is>
+      </c>
+      <c r="B31" s="27" t="inlineStr">
+        <is>
+          <t>Circuit Breaker</t>
+        </is>
+      </c>
+      <c r="C31" s="28" t="inlineStr">
+        <is>
+          <t>Verify Circuit Tripping from CLOSED to OPEN State upon Consecutive Provider Failures.</t>
+        </is>
+      </c>
+      <c r="D31" s="28" t="inlineStr">
+        <is>
+          <t>Active Circuit Breaker policy with threshold = 3.</t>
+        </is>
+      </c>
+      <c r="E31" s="28" t="inlineStr">
+        <is>
+          <t>1. Simulate 3 consecutive 503 Service Unavailable errors on Primary Provider.
+2. Observe dashboard state and send 4th request.</t>
+        </is>
+      </c>
+      <c r="F31" s="28" t="inlineStr">
+        <is>
+          <t>Errors: 3 consecutive HTTP 503 from Primary</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="inlineStr">
+        <is>
+          <t>Circuit breaker state immediately transitions to 'OPEN (Tripped / Red)'; 4th request is instantly rerouted to Fallback Provider without hitting dead primary; zero user timeout.</t>
+        </is>
+      </c>
+      <c r="H31" s="28" t="inlineStr">
+        <is>
+          <t>State transition CLOSED -&gt; OPEN verified. Fallback executed in &lt;5ms.</t>
+        </is>
+      </c>
+      <c r="I31" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J31" s="30" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K31" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L31" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M31" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="54" customHeight="1">
+      <c r="A32" s="26" t="inlineStr">
+        <is>
+          <t>TC_CB_03</t>
+        </is>
+      </c>
+      <c r="B32" s="27" t="inlineStr">
+        <is>
+          <t>Circuit Breaker</t>
+        </is>
+      </c>
+      <c r="C32" s="28" t="inlineStr">
+        <is>
+          <t>Verify HALF-OPEN Probe Evaluation and Automatic Recovery back to CLOSED State.</t>
+        </is>
+      </c>
+      <c r="D32" s="28" t="inlineStr">
+        <is>
+          <t>Circuit breaker is in OPEN state with 30s cooldown.</t>
+        </is>
+      </c>
+      <c r="E32" s="28" t="inlineStr">
+        <is>
+          <t>1. Wait 30 seconds for cooldown window to elapse.
+2. Observe state change to 'HALF-OPEN (Yellow)'.
+3. Send 1 probe request.
+4. Simulate upstream primary provider returning HTTP 200 OK.</t>
+        </is>
+      </c>
+      <c r="F32" s="28" t="inlineStr">
+        <is>
+          <t>State: OPEN -&gt; wait 30s -&gt; HALF-OPEN
+Probe request: Returns 200 OK</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="inlineStr">
+        <is>
+          <t>Probe request succeeds; circuit breaker detects primary recovery; state automatically resets to 'CLOSED (Normal / Green)'; normal routing restored.</t>
+        </is>
+      </c>
+      <c r="H32" s="28" t="inlineStr">
+        <is>
+          <t>Auto-recovery loop validated. Primary provider reinstated smoothly.</t>
+        </is>
+      </c>
+      <c r="I32" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J32" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K32" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L32" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M32" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="54" customHeight="1">
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t>TC_CB_04</t>
+        </is>
+      </c>
+      <c r="B33" s="27" t="inlineStr">
+        <is>
+          <t>Circuit Breaker</t>
+        </is>
+      </c>
+      <c r="C33" s="28" t="inlineStr">
+        <is>
+          <t>Verify Manual Circuit Reset from Admin Dashboard.</t>
+        </is>
+      </c>
+      <c r="D33" s="28" t="inlineStr">
+        <is>
+          <t>Circuit breaker is currently in OPEN or HALF-OPEN state.</t>
+        </is>
+      </c>
+      <c r="E33" s="28" t="inlineStr">
+        <is>
+          <t>1. Navigate to /workspace/circuit-breaker.
+2. Locate tripped breaker 'OpenAI-Resilience-Breaker'.
+3. Click 'Reset Circuit' action button.
+4. Confirm prompt.</t>
+        </is>
+      </c>
+      <c r="F33" s="28" t="inlineStr">
+        <is>
+          <t>Action: Click 'Reset Circuit' button</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="inlineStr">
+        <is>
+          <t>Circuit state immediately forces reset to 'CLOSED'; failure counters zeroed; toast confirms 'Circuit Breaker successfully reset'.</t>
+        </is>
+      </c>
+      <c r="H33" s="28" t="inlineStr">
+        <is>
+          <t>Manual reset command accepted; state restored to CLOSED.</t>
+        </is>
+      </c>
+      <c r="I33" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J33" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K33" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L33" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M33" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="26" customHeight="1">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
+          <t>SECTION 7: PRICING OVERRIDES &amp; TOKEN COST MANAGEMENT (/workspace/custom-pricing/overrides)</t>
+        </is>
+      </c>
+      <c r="B35" s="25" t="n"/>
+      <c r="C35" s="25" t="n"/>
+      <c r="D35" s="25" t="n"/>
+      <c r="E35" s="25" t="n"/>
+      <c r="F35" s="25" t="n"/>
+      <c r="G35" s="25" t="n"/>
+      <c r="H35" s="25" t="n"/>
+      <c r="I35" s="25" t="n"/>
+      <c r="J35" s="25" t="n"/>
+      <c r="K35" s="25" t="n"/>
+      <c r="L35" s="25" t="n"/>
+      <c r="M35" s="25" t="n"/>
+    </row>
+    <row r="36" ht="54" customHeight="1">
+      <c r="A36" s="26" t="inlineStr">
+        <is>
+          <t>TC_PRICE_01</t>
+        </is>
+      </c>
+      <c r="B36" s="27" t="inlineStr">
+        <is>
+          <t>Pricing Overrides</t>
+        </is>
+      </c>
+      <c r="C36" s="28" t="inlineStr">
+        <is>
+          <t>Create Custom Input &amp; Output Token Pricing Override per 1M Tokens for specific model.</t>
+        </is>
+      </c>
+      <c r="D36" s="28" t="inlineStr">
+        <is>
+          <t>Admin on https://unifai.yespanchi.com/workspace/custom-pricing/overrides.</t>
+        </is>
+      </c>
+      <c r="E36" s="28" t="inlineStr">
+        <is>
+          <t>1. Click 'Add Pricing Override' button.
+2. Select Scope: Model 'gpt-4o'.
+3. Enter Custom Input Token Price: $2.50 per 1M tokens ($0.0000025 / token).
+4. Enter Custom Output Token Price: $10.00 per 1M tokens ($0.0000100 / token).
+5. Currency: USD ($).
+6. Click 'Save Override'.</t>
+        </is>
+      </c>
+      <c r="F36" s="28" t="inlineStr">
+        <is>
+          <t>Model: gpt-4o
+Input: $2.50 / 1M
+Output: $10.00 / 1M
+Currency: USD</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="inlineStr">
+        <is>
+          <t>Pricing override saved; appears in Pricing Overrides table with 'Custom Active' badge; effective price reflected immediately.</t>
+        </is>
+      </c>
+      <c r="H36" s="28" t="inlineStr">
+        <is>
+          <t>Custom pricing record saved to database; cache invalidated.</t>
+        </is>
+      </c>
+      <c r="I36" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J36" s="30" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K36" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L36" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M36" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="54" customHeight="1">
+      <c r="A37" s="26" t="inlineStr">
+        <is>
+          <t>TC_PRICE_02</t>
+        </is>
+      </c>
+      <c r="B37" s="27" t="inlineStr">
+        <is>
+          <t>Pricing Overrides</t>
+        </is>
+      </c>
+      <c r="C37" s="28" t="inlineStr">
+        <is>
+          <t>Verify Real-time Chat Request Cost Calculation in Logs matches Custom Overrides.</t>
+        </is>
+      </c>
+      <c r="D37" s="28" t="inlineStr">
+        <is>
+          <t>Active pricing override: Input=$2.50/1M, Output=$10.00/1M for gpt-4o.</t>
+        </is>
+      </c>
+      <c r="E37" s="28" t="inlineStr">
+        <is>
+          <t>1. Send chat completion request via gateway with model 'gpt-4o'.
+2. Upstream returns: 2,000 prompt tokens, 1,000 completion tokens.
+3. Navigate to /workspace/logs and inspect request detail.
+4. Calculate expected: (2,000 * 0.0000025) + (1,000 * 0.00001) = $0.005 + $0.010 = $0.01500.</t>
+        </is>
+      </c>
+      <c r="F37" s="28" t="inlineStr">
+        <is>
+          <t>Prompt tokens: 2,000
+Completion tokens: 1,000
+Expected Cost: $0.015000</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="inlineStr">
+        <is>
+          <t>Log entry displays exact Total Cost: '$0.015000'; prompt cost and completion cost breakdown match custom override rates verbatim.</t>
+        </is>
+      </c>
+      <c r="H37" s="28" t="inlineStr">
+        <is>
+          <t>Cost arithmetic verified against custom override rates. Exact match.</t>
+        </is>
+      </c>
+      <c r="I37" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J37" s="30" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K37" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L37" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M37" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="54" customHeight="1">
+      <c r="A38" s="26" t="inlineStr">
+        <is>
+          <t>TC_PRICE_03</t>
+        </is>
+      </c>
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t>Pricing Overrides</t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="inlineStr">
+        <is>
+          <t>Scope-Based Pricing Override for Virtual Key (e.g. Enterprise Client Discount Tier).</t>
+        </is>
+      </c>
+      <c r="D38" s="28" t="inlineStr">
+        <is>
+          <t>Virtual Key 'VK-ENTERPRISE-CLIENT' exists in workspace.</t>
+        </is>
+      </c>
+      <c r="E38" s="28" t="inlineStr">
+        <is>
+          <t>1. Create Pricing Override with Scope: 'Virtual Key'.
+2. Select Virtual Key: 'VK-ENTERPRISE-CLIENT'.
+3. Set Negotiated Rate: Input $1.50/1M, Output $6.00/1M.
+4. Send request using this Virtual Key vs standard key.</t>
+        </is>
+      </c>
+      <c r="F38" s="28" t="inlineStr">
+        <is>
+          <t>Scope: Virtual Key (VK-ENTERPRISE-CLIENT)
+Input: $1.50/1M, Output: $6.00/1M</t>
+        </is>
+      </c>
+      <c r="G38" s="28" t="inlineStr">
+        <is>
+          <t>Requests with VK-ENTERPRISE-CLIENT are billed at discounted rates ($1.50/$6.00); all other keys continue to use global pricing.</t>
+        </is>
+      </c>
+      <c r="H38" s="28" t="inlineStr">
+        <is>
+          <t>Scoped virtual key override verified; isolation between keys confirmed.</t>
+        </is>
+      </c>
+      <c r="I38" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J38" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K38" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L38" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M38" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="54" customHeight="1">
+      <c r="A39" s="26" t="inlineStr">
+        <is>
+          <t>TC_PRICE_04</t>
+        </is>
+      </c>
+      <c r="B39" s="27" t="inlineStr">
+        <is>
+          <t>Pricing Overrides</t>
+        </is>
+      </c>
+      <c r="C39" s="28" t="inlineStr">
+        <is>
+          <t>Delete Pricing Override and verify automatic fallback to Standard Catalog Rates.</t>
+        </is>
+      </c>
+      <c r="D39" s="28" t="inlineStr">
+        <is>
+          <t>Custom pricing override active for gpt-4o.</t>
+        </is>
+      </c>
+      <c r="E39" s="28" t="inlineStr">
+        <is>
+          <t>1. In Pricing Overrides table, click 'Delete' on gpt-4o override.
+2. Confirm deletion.
+3. Send test request with 1,000 prompt tokens.</t>
+        </is>
+      </c>
+      <c r="F39" s="28" t="inlineStr">
+        <is>
+          <t>Action: Delete override for gpt-4o</t>
+        </is>
+      </c>
+      <c r="G39" s="28" t="inlineStr">
+        <is>
+          <t>Override removed; cost calculation seamlessly falls back to standard vendor catalog price ($5.00/1M input); zero errors.</t>
+        </is>
+      </c>
+      <c r="H39" s="28" t="inlineStr">
+        <is>
+          <t>Fallback to base catalog price verified after override removal.</t>
+        </is>
+      </c>
+      <c r="I39" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J39" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K39" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L39" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M39" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="26" customHeight="1">
+      <c r="A41" s="24" t="inlineStr">
+        <is>
+          <t>SECTION 8: GLOBAL MODEL SETTINGS &amp; ENGINE CONFIGURATION (/workspace/custom-pricing)</t>
+        </is>
+      </c>
+      <c r="B41" s="25" t="n"/>
+      <c r="C41" s="25" t="n"/>
+      <c r="D41" s="25" t="n"/>
+      <c r="E41" s="25" t="n"/>
+      <c r="F41" s="25" t="n"/>
+      <c r="G41" s="25" t="n"/>
+      <c r="H41" s="25" t="n"/>
+      <c r="I41" s="25" t="n"/>
+      <c r="J41" s="25" t="n"/>
+      <c r="K41" s="25" t="n"/>
+      <c r="L41" s="25" t="n"/>
+      <c r="M41" s="25" t="n"/>
+    </row>
+    <row r="42" ht="54" customHeight="1">
+      <c r="A42" s="26" t="inlineStr">
+        <is>
+          <t>TC_SETTING_01</t>
+        </is>
+      </c>
+      <c r="B42" s="27" t="inlineStr">
+        <is>
+          <t>Model Settings</t>
+        </is>
+      </c>
+      <c r="C42" s="28" t="inlineStr">
+        <is>
+          <t>Configure Global Default Model Parameters (Temperature, Max Output Tokens, Top-P).</t>
+        </is>
+      </c>
+      <c r="D42" s="28" t="inlineStr">
+        <is>
+          <t>Admin on https://unifai.yespanchi.com/workspace/custom-pricing.</t>
+        </is>
+      </c>
+      <c r="E42" s="28" t="inlineStr">
+        <is>
+          <t>1. Set Default Temperature: 0.7.
+2. Set Default Max Tokens: 4,096.
+3. Set Default Top-P: 0.95.
+4. Click 'Save Global Model Settings'.
+5. Send API request with no temperature specified.</t>
+        </is>
+      </c>
+      <c r="F42" s="28" t="inlineStr">
+        <is>
+          <t>Temperature: 0.7
+Max Tokens: 4096
+Top-P: 0.95</t>
+        </is>
+      </c>
+      <c r="G42" s="28" t="inlineStr">
+        <is>
+          <t>Global settings saved; gateway automatically injects temperature=0.7 and max_tokens=4096 into upstream payload when client omits them.</t>
+        </is>
+      </c>
+      <c r="H42" s="28" t="inlineStr">
+        <is>
+          <t>Payload inspection verified injection of global defaults.</t>
+        </is>
+      </c>
+      <c r="I42" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J42" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K42" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L42" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M42" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="54" customHeight="1">
+      <c r="A43" s="26" t="inlineStr">
+        <is>
+          <t>TC_SETTING_02</t>
+        </is>
+      </c>
+      <c r="B43" s="27" t="inlineStr">
+        <is>
+          <t>Model Settings</t>
+        </is>
+      </c>
+      <c r="C43" s="28" t="inlineStr">
+        <is>
+          <t>Configure Gateway Request Timeout &amp; Exponential Backoff Retry Strategy.</t>
+        </is>
+      </c>
+      <c r="D43" s="28" t="inlineStr">
+        <is>
+          <t>Admin on Model Settings page.</t>
+        </is>
+      </c>
+      <c r="E43" s="28" t="inlineStr">
+        <is>
+          <t>1. Set Gateway Upstream Timeout: 30 seconds.
+2. Set Max Automatic Retries: 3.
+3. Set Retry Backoff Multiplier: 1.5x.
+4. Click 'Save Settings'.
+5. Simulate slow provider response taking 35 seconds.</t>
+        </is>
+      </c>
+      <c r="F43" s="28" t="inlineStr">
+        <is>
+          <t>Timeout: 30s
+Retries: 3
+Backoff: 1.5x</t>
+        </is>
+      </c>
+      <c r="G43" s="28" t="inlineStr">
+        <is>
+          <t>Gateway cleanly terminates hanging request at exactly 30s; initiates retry 1 at 1.5s; succeeds or cascades to fallback cleanly without thread lock.</t>
+        </is>
+      </c>
+      <c r="H43" s="28" t="inlineStr">
+        <is>
+          <t>Timeout threshold and retry count verified under simulated latency.</t>
+        </is>
+      </c>
+      <c r="I43" s="29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J43" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K43" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L43" s="27" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="M43" s="27" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A19:M19"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A9:M9"/>
+    <mergeCell ref="A35:M35"/>
+    <mergeCell ref="A41:M41"/>
+    <mergeCell ref="A29:M29"/>
+    <mergeCell ref="A24:M24"/>
+    <mergeCell ref="A2:M2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>

</xml_diff>